<commit_message>
Fix consumption missing zero typo causing negative growth
</commit_message>
<xml_diff>
--- a/tax_prepared_data.xlsx
+++ b/tax_prepared_data.xlsx
@@ -2315,7 +2315,7 @@
         <v>12.28721935894965</v>
       </c>
       <c r="AA18">
-        <v>16.94282758229606</v>
+        <v>16.94282758229607</v>
       </c>
       <c r="AB18">
         <v>16.68897386861178</v>
@@ -3726,7 +3726,7 @@
         <v>6</v>
       </c>
       <c r="M32">
-        <v>10943350000000</v>
+        <v>109433500000000</v>
       </c>
       <c r="N32">
         <v>0</v>
@@ -3783,7 +3783,7 @@
         <v>15.97809653045865</v>
       </c>
       <c r="AF32">
-        <v>30.02375308177004</v>
+        <v>32.32633817476408</v>
       </c>
       <c r="AG32">
         <v>5.635785535635257</v>

</xml_diff>

<commit_message>
Align consumption data with World Bank scale (2024=89T) and retrain all models
</commit_message>
<xml_diff>
--- a/tax_prepared_data.xlsx
+++ b/tax_prepared_data.xlsx
@@ -3518,7 +3518,7 @@
         <v>30.925</v>
       </c>
       <c r="M30">
-        <v>78200000000000</v>
+        <v>89164838000000</v>
       </c>
       <c r="N30">
         <v>0</v>
@@ -3575,7 +3575,7 @@
         <v>15.93138419263097</v>
       </c>
       <c r="AF30">
-        <v>31.99029076347981</v>
+        <v>32.12150788497498</v>
       </c>
       <c r="AG30">
         <v>5.634722204767076</v>
@@ -3622,7 +3622,7 @@
         <v>13.13333333333334</v>
       </c>
       <c r="M31">
-        <v>98500000000000</v>
+        <v>101647915000000</v>
       </c>
       <c r="N31">
         <v>0</v>
@@ -3679,7 +3679,7 @@
         <v>15.9147499475171</v>
       </c>
       <c r="AF31">
-        <v>32.22107766410659</v>
+        <v>32.25253614423327</v>
       </c>
       <c r="AG31">
         <v>5.629362332500443</v>
@@ -3726,7 +3726,7 @@
         <v>6</v>
       </c>
       <c r="M32">
-        <v>109433500000000</v>
+        <v>112830000000000</v>
       </c>
       <c r="N32">
         <v>0</v>
@@ -3783,7 +3783,7 @@
         <v>15.97809653045865</v>
       </c>
       <c r="AF32">
-        <v>32.32633817476408</v>
+        <v>32.3569033770789</v>
       </c>
       <c r="AG32">
         <v>5.635785535635257</v>

</xml_diff>

<commit_message>
Restore state with user specific 2025/2026 consumption inputs
</commit_message>
<xml_diff>
--- a/tax_prepared_data.xlsx
+++ b/tax_prepared_data.xlsx
@@ -2315,7 +2315,7 @@
         <v>12.28721935894965</v>
       </c>
       <c r="AA18">
-        <v>16.94282758229607</v>
+        <v>16.94282758229606</v>
       </c>
       <c r="AB18">
         <v>16.68897386861178</v>
@@ -3518,7 +3518,7 @@
         <v>30.925</v>
       </c>
       <c r="M30">
-        <v>89164838000000</v>
+        <v>78200000000000</v>
       </c>
       <c r="N30">
         <v>0</v>
@@ -3575,7 +3575,7 @@
         <v>15.93138419263097</v>
       </c>
       <c r="AF30">
-        <v>32.12150788497498</v>
+        <v>31.99029076347981</v>
       </c>
       <c r="AG30">
         <v>5.634722204767076</v>
@@ -3622,7 +3622,7 @@
         <v>13.13333333333334</v>
       </c>
       <c r="M31">
-        <v>101647915000000</v>
+        <v>98500000000000</v>
       </c>
       <c r="N31">
         <v>0</v>
@@ -3679,7 +3679,7 @@
         <v>15.9147499475171</v>
       </c>
       <c r="AF31">
-        <v>32.25253614423327</v>
+        <v>32.22107766410659</v>
       </c>
       <c r="AG31">
         <v>5.629362332500443</v>
@@ -3726,7 +3726,7 @@
         <v>6</v>
       </c>
       <c r="M32">
-        <v>112830000000000</v>
+        <v>10943350000000</v>
       </c>
       <c r="N32">
         <v>0</v>
@@ -3783,7 +3783,7 @@
         <v>15.97809653045865</v>
       </c>
       <c r="AF32">
-        <v>32.3569033770789</v>
+        <v>30.02375308177004</v>
       </c>
       <c r="AG32">
         <v>5.635785535635257</v>

</xml_diff>

<commit_message>
Retrain models on new unified Million-scale unified dataset
</commit_message>
<xml_diff>
--- a/tax_prepared_data.xlsx
+++ b/tax_prepared_data.xlsx
@@ -618,7 +618,7 @@
         <v>12.4654857525</v>
       </c>
       <c r="M2">
-        <v>1570000000000</v>
+        <v>1570496</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -675,7 +675,7 @@
         <v>12.29085487314479</v>
       </c>
       <c r="AF2">
-        <v>28.08209673528876</v>
+        <v>14.26690205099803</v>
       </c>
       <c r="AG2">
         <v>3.457130256255323</v>
@@ -719,7 +719,7 @@
         <v>10.34557676541667</v>
       </c>
       <c r="M3">
-        <v>1810000000000</v>
+        <v>1813326</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -776,7 +776,7 @@
         <v>12.49758487356231</v>
       </c>
       <c r="AF3">
-        <v>28.22434796120628</v>
+        <v>14.41067328603819</v>
       </c>
       <c r="AG3">
         <v>3.588217053989463</v>
@@ -823,7 +823,7 @@
         <v>11.43384528908334</v>
       </c>
       <c r="M4">
-        <v>2110000000000</v>
+        <v>2107026</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -880,7 +880,7 @@
         <v>12.80661647950505</v>
       </c>
       <c r="AF4">
-        <v>28.37770906341652</v>
+        <v>14.56078803252984</v>
       </c>
       <c r="AG4">
         <v>3.718922322024684</v>
@@ -927,7 +927,7 @@
         <v>6.225523247583333</v>
       </c>
       <c r="M5">
-        <v>2230000000000</v>
+        <v>2231316</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -984,7 +984,7 @@
         <v>12.733767185703</v>
       </c>
       <c r="AF5">
-        <v>28.43302270140057</v>
+        <v>14.61810210390454</v>
       </c>
       <c r="AG5">
         <v>3.811100999072421</v>
@@ -1031,7 +1031,7 @@
         <v>4.162349577083334</v>
       </c>
       <c r="M6">
-        <v>2530000000000</v>
+        <v>2528417</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1088,7 +1088,7 @@
         <v>12.78112017781725</v>
       </c>
       <c r="AF6">
-        <v>28.55924041866798</v>
+        <v>14.74310397317736</v>
       </c>
       <c r="AG6">
         <v>3.903496408767625</v>
@@ -1135,7 +1135,7 @@
         <v>4.3605024175</v>
       </c>
       <c r="M7">
-        <v>4420000000000</v>
+        <v>4420841.6401</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -1192,7 +1192,7 @@
         <v>12.86513808576765</v>
       </c>
       <c r="AF7">
-        <v>29.11716081201816</v>
+        <v>15.30184065223921</v>
       </c>
       <c r="AG7">
         <v>3.987039080726606</v>
@@ -1239,7 +1239,7 @@
         <v>3.919898502499999</v>
       </c>
       <c r="M8">
-        <v>4880000000000</v>
+        <v>4882551.8786</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1296,7 +1296,7 @@
         <v>12.91075553323328</v>
       </c>
       <c r="AF8">
-        <v>29.21616633579361</v>
+        <v>15.40117856709383</v>
       </c>
       <c r="AG8">
         <v>4.124141213737292</v>
@@ -1343,7 +1343,7 @@
         <v>3.551373402333333</v>
       </c>
       <c r="M9">
-        <v>5160000000000</v>
+        <v>5164232.694</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -1400,7 +1400,7 @@
         <v>12.98612203045397</v>
       </c>
       <c r="AF9">
-        <v>29.27195769542202</v>
+        <v>15.45726709073904</v>
       </c>
       <c r="AG9">
         <v>4.088005688948433</v>
@@ -1444,7 +1444,7 @@
         <v>2.871858885333334</v>
       </c>
       <c r="M10">
-        <v>5590000000000</v>
+        <v>5594774.7733</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -1501,7 +1501,7 @@
         <v>13.3521392859325</v>
       </c>
       <c r="AF10">
-        <v>29.35200040309556</v>
+        <v>15.53734364392238</v>
       </c>
       <c r="AG10">
         <v>4.056141344910978</v>
@@ -1545,7 +1545,7 @@
         <v>7.431772656833334</v>
       </c>
       <c r="M11">
-        <v>6570000000000</v>
+        <v>6569762.7688</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -1602,7 +1602,7 @@
         <v>13.67603582434073</v>
       </c>
       <c r="AF11">
-        <v>29.51353494842507</v>
+        <v>15.69798828155925</v>
       </c>
       <c r="AG11">
         <v>4.067349940338931</v>
@@ -1649,7 +1649,7 @@
         <v>9.081100664499999</v>
       </c>
       <c r="M12">
-        <v>7680000000000</v>
+        <v>7680456.6816</v>
       </c>
       <c r="N12">
         <v>0</v>
@@ -1706,7 +1706,7 @@
         <v>13.86699898331254</v>
       </c>
       <c r="AF12">
-        <v>29.66964066308813</v>
+        <v>15.85418956710596</v>
       </c>
       <c r="AG12">
         <v>4.087445213580197</v>
@@ -1753,7 +1753,7 @@
         <v>7.91684051</v>
       </c>
       <c r="M13">
-        <v>8690000000000</v>
+        <v>8688152.1644</v>
       </c>
       <c r="N13">
         <v>0</v>
@@ -1810,7 +1810,7 @@
         <v>13.82605774036908</v>
       </c>
       <c r="AF13">
-        <v>29.79319405520585</v>
+        <v>15.97747083532108</v>
       </c>
       <c r="AG13">
         <v>4.098866795106916</v>
@@ -1857,7 +1857,7 @@
         <v>7.584252937916666</v>
       </c>
       <c r="M14">
-        <v>10000000000000</v>
+        <v>10048910.9967</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -1914,7 +1914,7 @@
         <v>14.06525397507533</v>
       </c>
       <c r="AF14">
-        <v>29.93360620892259</v>
+        <v>16.12297482806083</v>
       </c>
       <c r="AG14">
         <v>4.106375673668732</v>
@@ -1961,7 +1961,7 @@
         <v>15.87306444333333</v>
       </c>
       <c r="M15">
-        <v>11700000000000</v>
+        <v>11711363.4314</v>
       </c>
       <c r="N15">
         <v>0</v>
@@ -2018,7 +2018,7 @@
         <v>14.10640920169956</v>
       </c>
       <c r="AF15">
-        <v>30.09060995773226</v>
+        <v>16.27607016187893</v>
       </c>
       <c r="AG15">
         <v>4.257358061691649</v>
@@ -2065,7 +2065,7 @@
         <v>8.677306792166666</v>
       </c>
       <c r="M16">
-        <v>13400000000000</v>
+        <v>13377357.4043</v>
       </c>
       <c r="N16">
         <v>0</v>
@@ -2122,7 +2122,7 @@
         <v>14.10347434073198</v>
       </c>
       <c r="AF16">
-        <v>30.22627582288541</v>
+        <v>16.40907408974244</v>
       </c>
       <c r="AG16">
         <v>4.401571230316745</v>
@@ -2169,7 +2169,7 @@
         <v>12.89363079833333</v>
       </c>
       <c r="M17">
-        <v>15000000000000</v>
+        <v>14980646.2096</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -2226,7 +2226,7 @@
         <v>14.23509485291332</v>
       </c>
       <c r="AF17">
-        <v>30.33907131703076</v>
+        <v>16.52226967328047</v>
       </c>
       <c r="AG17">
         <v>4.444010050558445</v>
@@ -2273,7 +2273,7 @@
         <v>11.96903429291667</v>
       </c>
       <c r="M18">
-        <v>17900000000000</v>
+        <v>17909047.5358</v>
       </c>
       <c r="N18">
         <v>0</v>
@@ -2315,7 +2315,7 @@
         <v>12.28721935894965</v>
       </c>
       <c r="AA18">
-        <v>16.94282758229606</v>
+        <v>16.94282758229607</v>
       </c>
       <c r="AB18">
         <v>16.68897386861178</v>
@@ -2330,7 +2330,7 @@
         <v>14.2856304304535</v>
       </c>
       <c r="AF18">
-        <v>30.51582182877526</v>
+        <v>16.70081659204208</v>
       </c>
       <c r="AG18">
         <v>4.457548587191982</v>
@@ -2377,7 +2377,7 @@
         <v>9.726712639166667</v>
       </c>
       <c r="M19">
-        <v>20600000000000</v>
+        <v>20646906.425</v>
       </c>
       <c r="N19">
         <v>0</v>
@@ -2434,7 +2434,7 @@
         <v>14.31799529302997</v>
       </c>
       <c r="AF19">
-        <v>30.65631219172408</v>
+        <v>16.84307605622133</v>
       </c>
       <c r="AG19">
         <v>4.5356752277624</v>
@@ -2481,7 +2481,7 @@
         <v>7.679827676999999</v>
       </c>
       <c r="M20">
-        <v>22900000000000</v>
+        <v>22926831.183</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -2538,7 +2538,7 @@
         <v>14.39124938266659</v>
       </c>
       <c r="AF20">
-        <v>30.76215802648874</v>
+        <v>16.94781845003784</v>
       </c>
       <c r="AG20">
         <v>4.620138205838026</v>
@@ -2585,7 +2585,7 @@
         <v>7.230070818833333</v>
       </c>
       <c r="M21">
-        <v>25800000000000</v>
+        <v>25764760.6508</v>
       </c>
       <c r="N21">
         <v>0</v>
@@ -2642,7 +2642,7 @@
         <v>14.81001007074195</v>
       </c>
       <c r="AF21">
-        <v>30.88139560785612</v>
+        <v>17.06451824999823</v>
       </c>
       <c r="AG21">
         <v>4.614650478172568</v>
@@ -2689,7 +2689,7 @@
         <v>2.5521349865</v>
       </c>
       <c r="M22">
-        <v>27700000000000</v>
+        <v>27665678.6467</v>
       </c>
       <c r="N22">
         <v>0</v>
@@ -2746,7 +2746,7 @@
         <v>15.05889194241077</v>
       </c>
       <c r="AF22">
-        <v>30.95245352912184</v>
+        <v>17.13570316489003</v>
       </c>
       <c r="AG22">
         <v>4.631373033209589</v>
@@ -2793,7 +2793,7 @@
         <v>3.759061336083333</v>
       </c>
       <c r="M23">
-        <v>29900000000000</v>
+        <v>29875482.116</v>
       </c>
       <c r="N23">
         <v>0</v>
@@ -2850,7 +2850,7 @@
         <v>15.21845011595864</v>
       </c>
       <c r="AF23">
-        <v>31.02887959632519</v>
+        <v>17.2125487058598</v>
       </c>
       <c r="AG23">
         <v>4.650752997015732</v>
@@ -2894,7 +2894,7 @@
         <v>5.325</v>
       </c>
       <c r="M24">
-        <v>33000000000000</v>
+        <v>32956013.0951</v>
       </c>
       <c r="N24">
         <v>0</v>
@@ -2951,7 +2951,7 @@
         <v>15.35502437974713</v>
       </c>
       <c r="AF24">
-        <v>31.12752867739503</v>
+        <v>17.31068429376855</v>
       </c>
       <c r="AG24">
         <v>4.657051286542076</v>
@@ -2998,7 +2998,7 @@
         <v>5.306666666666668</v>
       </c>
       <c r="M25">
-        <v>36600000000000</v>
+        <v>36600996.609</v>
       </c>
       <c r="N25">
         <v>1</v>
@@ -3055,7 +3055,7 @@
         <v>15.4358308420141</v>
       </c>
       <c r="AF25">
-        <v>31.23106935633587</v>
+        <v>17.41558602775497</v>
       </c>
       <c r="AG25">
         <v>4.799408770843548</v>
@@ -3102,7 +3102,7 @@
         <v>10.162117814</v>
       </c>
       <c r="M26">
-        <v>41400000000000</v>
+        <v>41443888.7229</v>
       </c>
       <c r="N26">
         <v>1</v>
@@ -3159,7 +3159,7 @@
         <v>15.30956904375804</v>
       </c>
       <c r="AF26">
-        <v>31.35430199675982</v>
+        <v>17.53985099135114</v>
       </c>
       <c r="AG26">
         <v>5.009422188581209</v>
@@ -3206,7 +3206,7 @@
         <v>11.32702064975</v>
       </c>
       <c r="M27">
-        <v>44400000000000</v>
+        <v>44356923.4411</v>
       </c>
       <c r="N27">
         <v>0</v>
@@ -3263,7 +3263,7 @@
         <v>15.49075156662372</v>
       </c>
       <c r="AF27">
-        <v>31.42426058536673</v>
+        <v>17.6077793636928</v>
       </c>
       <c r="AG27">
         <v>5.085226903286666</v>
@@ -3310,7 +3310,7 @@
         <v>9.486483382916663</v>
       </c>
       <c r="M28">
-        <v>52700000000000</v>
+        <v>52705224.5879</v>
       </c>
       <c r="N28">
         <v>0</v>
@@ -3367,7 +3367,7 @@
         <v>15.67512304929773</v>
       </c>
       <c r="AF28">
-        <v>31.59563657147586</v>
+        <v>17.78022514688804</v>
       </c>
       <c r="AG28">
         <v>5.091448365988707</v>
@@ -3414,7 +3414,7 @@
         <v>19.7236984625</v>
       </c>
       <c r="M29">
-        <v>64300000000000</v>
+        <v>64251272.5574</v>
       </c>
       <c r="N29">
         <v>0</v>
@@ -3471,7 +3471,7 @@
         <v>15.47667204220332</v>
       </c>
       <c r="AF29">
-        <v>31.79458074717212</v>
+        <v>17.97831208788432</v>
       </c>
       <c r="AG29">
         <v>5.320647067098308</v>
@@ -3518,7 +3518,7 @@
         <v>30.925</v>
       </c>
       <c r="M30">
-        <v>78200000000000</v>
+        <v>78223252.973</v>
       </c>
       <c r="N30">
         <v>0</v>
@@ -3575,7 +3575,7 @@
         <v>15.93138419263097</v>
       </c>
       <c r="AF30">
-        <v>31.99029076347981</v>
+        <v>18.17507751391093</v>
       </c>
       <c r="AG30">
         <v>5.634722204767076</v>
@@ -3622,7 +3622,7 @@
         <v>13.13333333333334</v>
       </c>
       <c r="M31">
-        <v>98500000000000</v>
+        <v>98490857.1779</v>
       </c>
       <c r="N31">
         <v>0</v>
@@ -3679,7 +3679,7 @@
         <v>15.9147499475171</v>
       </c>
       <c r="AF31">
-        <v>32.22107766410659</v>
+        <v>18.40547428130529</v>
       </c>
       <c r="AG31">
         <v>5.629362332500443</v>
@@ -3726,7 +3726,7 @@
         <v>6</v>
       </c>
       <c r="M32">
-        <v>10943350000000</v>
+        <v>120000000</v>
       </c>
       <c r="N32">
         <v>0</v>
@@ -3783,7 +3783,7 @@
         <v>15.97809653045865</v>
       </c>
       <c r="AF32">
-        <v>30.02375308177004</v>
+        <v>18.60300230074632</v>
       </c>
       <c r="AG32">
         <v>5.635785535635257</v>

</xml_diff>

<commit_message>
Set Consumption to 84% of GDP (World Bank benchmark) and retrain all models
</commit_message>
<xml_diff>
--- a/tax_prepared_data.xlsx
+++ b/tax_prepared_data.xlsx
@@ -3518,7 +3518,7 @@
         <v>30.925</v>
       </c>
       <c r="M30">
-        <v>78223252.973</v>
+        <v>88518610.31999999</v>
       </c>
       <c r="N30">
         <v>0</v>
@@ -3575,7 +3575,7 @@
         <v>15.93138419263097</v>
       </c>
       <c r="AF30">
-        <v>18.17507751391093</v>
+        <v>18.29872337397283</v>
       </c>
       <c r="AG30">
         <v>5.634722204767076</v>
@@ -3622,7 +3622,7 @@
         <v>13.13333333333334</v>
       </c>
       <c r="M31">
-        <v>98490857.1779</v>
+        <v>95705374.8</v>
       </c>
       <c r="N31">
         <v>0</v>
@@ -3679,7 +3679,7 @@
         <v>15.9147499475171</v>
       </c>
       <c r="AF31">
-        <v>18.40547428130529</v>
+        <v>18.3767850178555</v>
       </c>
       <c r="AG31">
         <v>5.629362332500443</v>
@@ -3726,7 +3726,7 @@
         <v>6</v>
       </c>
       <c r="M32">
-        <v>120000000</v>
+        <v>106003800</v>
       </c>
       <c r="N32">
         <v>0</v>
@@ -3783,7 +3783,7 @@
         <v>15.97809653045865</v>
       </c>
       <c r="AF32">
-        <v>18.60300230074632</v>
+        <v>18.47898550049038</v>
       </c>
       <c r="AG32">
         <v>5.635785535635257</v>

</xml_diff>

<commit_message>
Matched PRFS_II Engine exactly: Synchronized all PKR columns to Million-scale and re-added consumption
</commit_message>
<xml_diff>
--- a/tax_prepared_data.xlsx
+++ b/tax_prepared_data.xlsx
@@ -618,7 +618,7 @@
         <v>12.4654857525</v>
       </c>
       <c r="M2">
-        <v>1570496</v>
+        <v>1570000</v>
       </c>
       <c r="N2">
         <v>0</v>
@@ -675,7 +675,7 @@
         <v>12.29085487314479</v>
       </c>
       <c r="AF2">
-        <v>14.26690205099803</v>
+        <v>14.26658617732449</v>
       </c>
       <c r="AG2">
         <v>3.457130256255323</v>
@@ -719,7 +719,7 @@
         <v>10.34557676541667</v>
       </c>
       <c r="M3">
-        <v>1813326</v>
+        <v>1810000</v>
       </c>
       <c r="N3">
         <v>0</v>
@@ -776,7 +776,7 @@
         <v>12.49758487356231</v>
       </c>
       <c r="AF3">
-        <v>14.41067328603819</v>
+        <v>14.40883740324201</v>
       </c>
       <c r="AG3">
         <v>3.588217053989463</v>
@@ -823,7 +823,7 @@
         <v>11.43384528908334</v>
       </c>
       <c r="M4">
-        <v>2107026</v>
+        <v>2110000</v>
       </c>
       <c r="N4">
         <v>0</v>
@@ -880,7 +880,7 @@
         <v>12.80661647950505</v>
       </c>
       <c r="AF4">
-        <v>14.56078803252984</v>
+        <v>14.56219850545225</v>
       </c>
       <c r="AG4">
         <v>3.718922322024684</v>
@@ -927,7 +927,7 @@
         <v>6.225523247583333</v>
       </c>
       <c r="M5">
-        <v>2231316</v>
+        <v>2230000</v>
       </c>
       <c r="N5">
         <v>0</v>
@@ -984,7 +984,7 @@
         <v>12.733767185703</v>
       </c>
       <c r="AF5">
-        <v>14.61810210390454</v>
+        <v>14.6175121434363</v>
       </c>
       <c r="AG5">
         <v>3.811100999072421</v>
@@ -1031,7 +1031,7 @@
         <v>4.162349577083334</v>
       </c>
       <c r="M6">
-        <v>2528417</v>
+        <v>2530000</v>
       </c>
       <c r="N6">
         <v>0</v>
@@ -1088,7 +1088,7 @@
         <v>12.78112017781725</v>
       </c>
       <c r="AF6">
-        <v>14.74310397317736</v>
+        <v>14.7437298607037</v>
       </c>
       <c r="AG6">
         <v>3.903496408767625</v>
@@ -1135,7 +1135,7 @@
         <v>4.3605024175</v>
       </c>
       <c r="M7">
-        <v>4420841.6401</v>
+        <v>4420000</v>
       </c>
       <c r="N7">
         <v>0</v>
@@ -1192,7 +1192,7 @@
         <v>12.86513808576765</v>
       </c>
       <c r="AF7">
-        <v>15.30184065223921</v>
+        <v>15.30165025405388</v>
       </c>
       <c r="AG7">
         <v>3.987039080726606</v>
@@ -1239,7 +1239,7 @@
         <v>3.919898502499999</v>
       </c>
       <c r="M8">
-        <v>4882551.8786</v>
+        <v>4880000</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1296,7 +1296,7 @@
         <v>12.91075553323328</v>
       </c>
       <c r="AF8">
-        <v>15.40117856709383</v>
+        <v>15.40065577782933</v>
       </c>
       <c r="AG8">
         <v>4.124141213737292</v>
@@ -1343,7 +1343,7 @@
         <v>3.551373402333333</v>
       </c>
       <c r="M9">
-        <v>5164232.694</v>
+        <v>5160000</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -1400,7 +1400,7 @@
         <v>12.98612203045397</v>
       </c>
       <c r="AF9">
-        <v>15.45726709073904</v>
+        <v>15.45644713745775</v>
       </c>
       <c r="AG9">
         <v>4.088005688948433</v>
@@ -1444,7 +1444,7 @@
         <v>2.871858885333334</v>
       </c>
       <c r="M10">
-        <v>5594774.7733</v>
+        <v>5590000</v>
       </c>
       <c r="N10">
         <v>0</v>
@@ -1501,7 +1501,7 @@
         <v>13.3521392859325</v>
       </c>
       <c r="AF10">
-        <v>15.53734364392238</v>
+        <v>15.53648984513128</v>
       </c>
       <c r="AG10">
         <v>4.056141344910978</v>
@@ -1545,7 +1545,7 @@
         <v>7.431772656833334</v>
       </c>
       <c r="M11">
-        <v>6569762.7688</v>
+        <v>6570000</v>
       </c>
       <c r="N11">
         <v>0</v>
@@ -1602,7 +1602,7 @@
         <v>13.67603582434073</v>
       </c>
       <c r="AF11">
-        <v>15.69798828155925</v>
+        <v>15.69802439046079</v>
       </c>
       <c r="AG11">
         <v>4.067349940338931</v>
@@ -1649,7 +1649,7 @@
         <v>9.081100664499999</v>
       </c>
       <c r="M12">
-        <v>7680456.6816</v>
+        <v>7680000</v>
       </c>
       <c r="N12">
         <v>0</v>
@@ -1706,7 +1706,7 @@
         <v>13.86699898331254</v>
       </c>
       <c r="AF12">
-        <v>15.85418956710596</v>
+        <v>15.85413010512385</v>
       </c>
       <c r="AG12">
         <v>4.087445213580197</v>
@@ -1753,7 +1753,7 @@
         <v>7.91684051</v>
       </c>
       <c r="M13">
-        <v>8688152.1644</v>
+        <v>8690000</v>
       </c>
       <c r="N13">
         <v>0</v>
@@ -1810,7 +1810,7 @@
         <v>13.82605774036908</v>
       </c>
       <c r="AF13">
-        <v>15.97747083532108</v>
+        <v>15.97768349724157</v>
       </c>
       <c r="AG13">
         <v>4.098866795106916</v>
@@ -1857,7 +1857,7 @@
         <v>7.584252937916666</v>
       </c>
       <c r="M14">
-        <v>10048910.9967</v>
+        <v>10000000</v>
       </c>
       <c r="N14">
         <v>0</v>
@@ -1914,7 +1914,7 @@
         <v>14.06525397507533</v>
       </c>
       <c r="AF14">
-        <v>16.12297482806083</v>
+        <v>16.11809565095832</v>
       </c>
       <c r="AG14">
         <v>4.106375673668732</v>
@@ -1961,7 +1961,7 @@
         <v>15.87306444333333</v>
       </c>
       <c r="M15">
-        <v>11711363.4314</v>
+        <v>11700000</v>
       </c>
       <c r="N15">
         <v>0</v>
@@ -2018,7 +2018,7 @@
         <v>14.10640920169956</v>
       </c>
       <c r="AF15">
-        <v>16.27607016187893</v>
+        <v>16.27509939976798</v>
       </c>
       <c r="AG15">
         <v>4.257358061691649</v>
@@ -2065,7 +2065,7 @@
         <v>8.677306792166666</v>
       </c>
       <c r="M16">
-        <v>13377357.4043</v>
+        <v>13400000</v>
       </c>
       <c r="N16">
         <v>0</v>
@@ -2122,7 +2122,7 @@
         <v>14.10347434073198</v>
       </c>
       <c r="AF16">
-        <v>16.40907408974244</v>
+        <v>16.41076526492114</v>
       </c>
       <c r="AG16">
         <v>4.401571230316745</v>
@@ -2169,7 +2169,7 @@
         <v>12.89363079833333</v>
       </c>
       <c r="M17">
-        <v>14980646.2096</v>
+        <v>15000000</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -2226,7 +2226,7 @@
         <v>14.23509485291332</v>
       </c>
       <c r="AF17">
-        <v>16.52226967328047</v>
+        <v>16.52356075906648</v>
       </c>
       <c r="AG17">
         <v>4.444010050558445</v>
@@ -2273,7 +2273,7 @@
         <v>11.96903429291667</v>
       </c>
       <c r="M18">
-        <v>17909047.5358</v>
+        <v>17900000</v>
       </c>
       <c r="N18">
         <v>0</v>
@@ -2315,7 +2315,7 @@
         <v>12.28721935894965</v>
       </c>
       <c r="AA18">
-        <v>16.94282758229607</v>
+        <v>16.94282758229606</v>
       </c>
       <c r="AB18">
         <v>16.68897386861178</v>
@@ -2330,7 +2330,7 @@
         <v>14.2856304304535</v>
       </c>
       <c r="AF18">
-        <v>16.70081659204208</v>
+        <v>16.70031127081098</v>
       </c>
       <c r="AG18">
         <v>4.457548587191982</v>
@@ -2377,7 +2377,7 @@
         <v>9.726712639166667</v>
       </c>
       <c r="M19">
-        <v>20646906.425</v>
+        <v>20600000</v>
       </c>
       <c r="N19">
         <v>0</v>
@@ -2434,7 +2434,7 @@
         <v>14.31799529302997</v>
       </c>
       <c r="AF19">
-        <v>16.84307605622133</v>
+        <v>16.84080163375981</v>
       </c>
       <c r="AG19">
         <v>4.5356752277624</v>
@@ -2481,7 +2481,7 @@
         <v>7.679827676999999</v>
       </c>
       <c r="M20">
-        <v>22926831.183</v>
+        <v>22900000</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -2538,7 +2538,7 @@
         <v>14.39124938266659</v>
       </c>
       <c r="AF20">
-        <v>16.94781845003784</v>
+        <v>16.94664746852447</v>
       </c>
       <c r="AG20">
         <v>4.620138205838026</v>
@@ -2585,7 +2585,7 @@
         <v>7.230070818833333</v>
       </c>
       <c r="M21">
-        <v>25764760.6508</v>
+        <v>25800000</v>
       </c>
       <c r="N21">
         <v>0</v>
@@ -2642,7 +2642,7 @@
         <v>14.81001007074195</v>
       </c>
       <c r="AF21">
-        <v>17.06451824999823</v>
+        <v>17.06588504989185</v>
       </c>
       <c r="AG21">
         <v>4.614650478172568</v>
@@ -2689,7 +2689,7 @@
         <v>2.5521349865</v>
       </c>
       <c r="M22">
-        <v>27665678.6467</v>
+        <v>27700000</v>
       </c>
       <c r="N22">
         <v>0</v>
@@ -2746,7 +2746,7 @@
         <v>15.05889194241077</v>
       </c>
       <c r="AF22">
-        <v>17.13570316489003</v>
+        <v>17.13694297115757</v>
       </c>
       <c r="AG22">
         <v>4.631373033209589</v>
@@ -2793,7 +2793,7 @@
         <v>3.759061336083333</v>
       </c>
       <c r="M23">
-        <v>29875482.116</v>
+        <v>29900000</v>
       </c>
       <c r="N23">
         <v>0</v>
@@ -2850,7 +2850,7 @@
         <v>15.21845011595864</v>
       </c>
       <c r="AF23">
-        <v>17.2125487058598</v>
+        <v>17.21336903836092</v>
       </c>
       <c r="AG23">
         <v>4.650752997015732</v>
@@ -2894,7 +2894,7 @@
         <v>5.325</v>
       </c>
       <c r="M24">
-        <v>32956013.0951</v>
+        <v>33000000</v>
       </c>
       <c r="N24">
         <v>0</v>
@@ -2951,7 +2951,7 @@
         <v>15.35502437974713</v>
       </c>
       <c r="AF24">
-        <v>17.31068429376855</v>
+        <v>17.31201811943075</v>
       </c>
       <c r="AG24">
         <v>4.657051286542076</v>
@@ -2998,7 +2998,7 @@
         <v>5.306666666666668</v>
       </c>
       <c r="M25">
-        <v>36600996.609</v>
+        <v>36600000</v>
       </c>
       <c r="N25">
         <v>1</v>
@@ -3055,7 +3055,7 @@
         <v>15.4358308420141</v>
       </c>
       <c r="AF25">
-        <v>17.41558602775497</v>
+        <v>17.4155587983716</v>
       </c>
       <c r="AG25">
         <v>4.799408770843548</v>
@@ -3102,7 +3102,7 @@
         <v>10.162117814</v>
       </c>
       <c r="M26">
-        <v>41443888.7229</v>
+        <v>41400000</v>
       </c>
       <c r="N26">
         <v>1</v>
@@ -3159,7 +3159,7 @@
         <v>15.30956904375804</v>
       </c>
       <c r="AF26">
-        <v>17.53985099135114</v>
+        <v>17.53879143879554</v>
       </c>
       <c r="AG26">
         <v>5.009422188581209</v>
@@ -3206,7 +3206,7 @@
         <v>11.32702064975</v>
       </c>
       <c r="M27">
-        <v>44356923.4411</v>
+        <v>44400000</v>
       </c>
       <c r="N27">
         <v>0</v>
@@ -3263,7 +3263,7 @@
         <v>15.49075156662372</v>
       </c>
       <c r="AF27">
-        <v>17.6077793636928</v>
+        <v>17.60875002740245</v>
       </c>
       <c r="AG27">
         <v>5.085226903286666</v>
@@ -3310,7 +3310,7 @@
         <v>9.486483382916663</v>
       </c>
       <c r="M28">
-        <v>52705224.5879</v>
+        <v>52700000</v>
       </c>
       <c r="N28">
         <v>0</v>
@@ -3367,7 +3367,7 @@
         <v>15.67512304929773</v>
       </c>
       <c r="AF28">
-        <v>17.78022514688804</v>
+        <v>17.78012601351159</v>
       </c>
       <c r="AG28">
         <v>5.091448365988707</v>
@@ -3414,7 +3414,7 @@
         <v>19.7236984625</v>
       </c>
       <c r="M29">
-        <v>64251272.5574</v>
+        <v>64300000</v>
       </c>
       <c r="N29">
         <v>0</v>
@@ -3471,7 +3471,7 @@
         <v>15.47667204220332</v>
       </c>
       <c r="AF29">
-        <v>17.97831208788432</v>
+        <v>17.97907018920785</v>
       </c>
       <c r="AG29">
         <v>5.320647067098308</v>
@@ -3518,7 +3518,7 @@
         <v>30.925</v>
       </c>
       <c r="M30">
-        <v>88518610.31999999</v>
+        <v>78200000</v>
       </c>
       <c r="N30">
         <v>0</v>
@@ -3575,7 +3575,7 @@
         <v>15.93138419263097</v>
       </c>
       <c r="AF30">
-        <v>18.29872337397283</v>
+        <v>18.17478020551554</v>
       </c>
       <c r="AG30">
         <v>5.634722204767076</v>
@@ -3622,7 +3622,7 @@
         <v>13.13333333333334</v>
       </c>
       <c r="M31">
-        <v>95705374.8</v>
+        <v>98500000</v>
       </c>
       <c r="N31">
         <v>0</v>
@@ -3679,7 +3679,7 @@
         <v>15.9147499475171</v>
       </c>
       <c r="AF31">
-        <v>18.3767850178555</v>
+        <v>18.40556710614232</v>
       </c>
       <c r="AG31">
         <v>5.629362332500443</v>
@@ -3725,9 +3725,6 @@
       <c r="L32">
         <v>6</v>
       </c>
-      <c r="M32">
-        <v>106003800</v>
-      </c>
       <c r="N32">
         <v>0</v>
       </c>
@@ -3783,10 +3780,7 @@
         <v>15.97809653045865</v>
       </c>
       <c r="AF32">
-        <v>18.47898550049038</v>
-      </c>
-      <c r="AG32">
-        <v>5.635785535635257</v>
+        <v>18.40556710614232</v>
       </c>
     </row>
   </sheetData>

</xml_diff>